<commit_message>
refactor: hapus tuntas sisa kode dan skema lama
</commit_message>
<xml_diff>
--- a/Data/Database_Stok_Segara_Dummy.xlsx
+++ b/Data/Database_Stok_Segara_Dummy.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -468,7 +468,6 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="21" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -527,16 +526,11 @@
           <t>catatan</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>opname_rekap</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>m1q1h2a</t>
+          <t>m10coly</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -577,12 +571,11 @@
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>m2ymdky</t>
+          <t>m2mu7n0</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -623,12 +616,11 @@
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>m3ojt68</t>
+          <t>m3vyiil</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -669,12 +661,11 @@
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>m4bo71q</t>
+          <t>m4lqzwv</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -715,12 +706,11 @@
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>m5o80zg</t>
+          <t>m57wr9j</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -761,12 +751,11 @@
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>m6bxcak</t>
+          <t>m6tp9v4</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -807,12 +796,11 @@
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>m7n4lou</t>
+          <t>m7j6k35</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -853,12 +841,11 @@
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>m8bd8ds</t>
+          <t>m8hz0u0</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -899,12 +886,11 @@
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>m9ka5wa</t>
+          <t>m9obd0s</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -945,12 +931,11 @@
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>ma2rn1e</t>
+          <t>mawsv08</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -991,12 +976,11 @@
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>mbkzgv3</t>
+          <t>mbpy3qx</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1037,12 +1021,11 @@
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>mcbd3eq</t>
+          <t>mc7puqh</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1083,12 +1066,11 @@
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr"/>
-      <c r="L13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>md9qr7l</t>
+          <t>mdu2xvh</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1129,12 +1111,11 @@
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr"/>
-      <c r="L14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>me7wzce</t>
+          <t>me3xemz</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1175,12 +1156,11 @@
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr"/>
-      <c r="L15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>mfwnv66</t>
+          <t>mfannts</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1221,12 +1201,11 @@
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr"/>
-      <c r="L16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>mgi1yel</t>
+          <t>mgmpkn5</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1267,12 +1246,11 @@
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr"/>
-      <c r="L17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>mhbbnvy</t>
+          <t>mhtq606</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1313,12 +1291,11 @@
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr"/>
-      <c r="L18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>miwyf2z</t>
+          <t>miofm01</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1359,12 +1336,11 @@
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr"/>
-      <c r="L19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>mjrgjxs</t>
+          <t>mjvyxzx</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1409,12 +1385,11 @@
           <t>1 Pack Isi 10 pcs</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>mkpyjnk</t>
+          <t>mkd0a8o</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1455,12 +1430,11 @@
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr"/>
-      <c r="L21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>mlj43j3</t>
+          <t>mlee570</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1501,12 +1475,11 @@
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr"/>
-      <c r="L22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>mmv05l4</t>
+          <t>mmzmhqu</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1547,7 +1520,6 @@
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr"/>
-      <c r="L23" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1594,7 +1566,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>mnej4gh</t>
+          <t>mn3kzj8</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -1614,7 +1586,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>molx3s9</t>
+          <t>mokej3l</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -1630,7 +1602,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>mp30vbe</t>
+          <t>mpe6o5u</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -1646,7 +1618,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>mqj3zen</t>
+          <t>mq8xtsq</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -1776,15 +1748,15 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>m2iyslm4</t>
+          <t>m2i22qc9</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>1790608311755</v>
+        <v>1790616184338</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>28/09/2026 22:11</t>
+          <t>29/09/2026 00:23</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1794,7 +1766,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>m1q1h2a</t>
+          <t>m10coly</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1807,7 +1779,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>mnej4gh</t>
+          <t>mn3kzj8</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -1846,15 +1818,15 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>m2j8rxa8</t>
+          <t>m2jw4cpc</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>1790608311755</v>
+        <v>1790616184338</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>28/09/2026 22:11</t>
+          <t>29/09/2026 00:23</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -1864,7 +1836,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>m2ymdky</t>
+          <t>m2mu7n0</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1877,7 +1849,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>mnej4gh</t>
+          <t>mn3kzj8</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -1916,15 +1888,15 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>m2ky762z</t>
+          <t>m2kylibm</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1790608311755</v>
+        <v>1790616184338</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>28/09/2026 22:11</t>
+          <t>29/09/2026 00:23</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -1934,7 +1906,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>m3ojt68</t>
+          <t>m3vyiil</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1947,7 +1919,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>mnej4gh</t>
+          <t>mn3kzj8</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -1986,15 +1958,15 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>m2lfn83q</t>
+          <t>m2lv69go</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>1790608311755</v>
+        <v>1790616184338</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>28/09/2026 22:11</t>
+          <t>29/09/2026 00:23</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -2004,7 +1976,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>m4bo71q</t>
+          <t>m4lqzwv</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -2017,7 +1989,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>mnej4gh</t>
+          <t>mn3kzj8</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -2056,7 +2028,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>m1y8vrs9</t>
+          <t>m1yjx81j</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -2074,7 +2046,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>m1q1h2a</t>
+          <t>m10coly</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -2087,7 +2059,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>mnej4gh</t>
+          <t>mn3kzj8</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -2126,7 +2098,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>m1zbgk22</t>
+          <t>m1zmxlxs</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
@@ -2144,7 +2116,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>m2ymdky</t>
+          <t>m2mu7n0</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -2157,7 +2129,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>mnej4gh</t>
+          <t>mn3kzj8</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -2196,7 +2168,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>m209nrmk</t>
+          <t>m20pen8h</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -2214,7 +2186,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>m3ojt68</t>
+          <t>m3vyiil</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -2227,7 +2199,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>mnej4gh</t>
+          <t>mn3kzj8</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -2266,7 +2238,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>m21vq14r</t>
+          <t>m21773um</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
@@ -2284,7 +2256,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>m4bo71q</t>
+          <t>m4lqzwv</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -2297,7 +2269,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>mnej4gh</t>
+          <t>mn3kzj8</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -2336,7 +2308,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>m223tuc6</t>
+          <t>m2234z2p</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -2354,7 +2326,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>m5o80zg</t>
+          <t>m57wr9j</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -2367,7 +2339,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>mnej4gh</t>
+          <t>mn3kzj8</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -2406,7 +2378,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>m23e4brg</t>
+          <t>m23i6im9</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
@@ -2424,7 +2396,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>m6bxcak</t>
+          <t>m6tp9v4</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -2437,7 +2409,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>mnej4gh</t>
+          <t>mn3kzj8</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -2476,7 +2448,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>m248g1nt</t>
+          <t>m24cj9ff</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -2494,7 +2466,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>m7n4lou</t>
+          <t>m7j6k35</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -2507,7 +2479,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>mnej4gh</t>
+          <t>mn3kzj8</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -2546,7 +2518,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>m255pq9r</t>
+          <t>m256yfuy</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
@@ -2564,7 +2536,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>m8bd8ds</t>
+          <t>m8hz0u0</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -2577,7 +2549,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>mnej4gh</t>
+          <t>mn3kzj8</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -2616,7 +2588,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>m26n18sz</t>
+          <t>m26k28av</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -2634,7 +2606,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>m9ka5wa</t>
+          <t>m9obd0s</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -2647,7 +2619,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>mnej4gh</t>
+          <t>mn3kzj8</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -2686,7 +2658,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>m27r8p2u</t>
+          <t>m271a894</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
@@ -2704,7 +2676,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>ma2rn1e</t>
+          <t>mawsv08</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -2717,7 +2689,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>mnej4gh</t>
+          <t>mn3kzj8</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -2756,7 +2728,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>m285jcql</t>
+          <t>m281jrmm</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -2774,7 +2746,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>mbkzgv3</t>
+          <t>mbpy3qx</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -2787,7 +2759,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>mnej4gh</t>
+          <t>mn3kzj8</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -2826,7 +2798,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>m29l9x7t</t>
+          <t>m29wykht</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
@@ -2844,7 +2816,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>mcbd3eq</t>
+          <t>mc7puqh</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -2857,7 +2829,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>mnej4gh</t>
+          <t>mn3kzj8</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -2896,7 +2868,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>m2axkxpf</t>
+          <t>m2ai5u3t</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -2914,7 +2886,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>md9qr7l</t>
+          <t>mdu2xvh</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -2927,7 +2899,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>mnej4gh</t>
+          <t>mn3kzj8</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -2966,7 +2938,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>m2bkabn9</t>
+          <t>m2bigyrt</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
@@ -2984,7 +2956,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>me7wzce</t>
+          <t>me3xemz</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -2997,7 +2969,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>mnej4gh</t>
+          <t>mn3kzj8</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -3036,7 +3008,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>m2ckx58o</t>
+          <t>m2cjpu7a</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -3054,7 +3026,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>mfwnv66</t>
+          <t>mfannts</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -3067,7 +3039,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>mnej4gh</t>
+          <t>mn3kzj8</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -3106,7 +3078,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>m2dgdoou</t>
+          <t>m2dhbamk</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
@@ -3124,7 +3096,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>mgi1yel</t>
+          <t>mgmpkn5</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -3137,7 +3109,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>mnej4gh</t>
+          <t>mn3kzj8</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -3176,7 +3148,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>m2e6aj9h</t>
+          <t>m2eeuzpi</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -3194,7 +3166,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>mhbbnvy</t>
+          <t>mhtq606</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -3207,7 +3179,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>mnej4gh</t>
+          <t>mn3kzj8</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -3246,7 +3218,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>m2f4xa9u</t>
+          <t>m2f5obz7</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
@@ -3264,7 +3236,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>miwyf2z</t>
+          <t>miofm01</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -3277,7 +3249,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>mnej4gh</t>
+          <t>mn3kzj8</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -3316,7 +3288,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>m2gondau</t>
+          <t>m2gndh9s</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -3334,7 +3306,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>mjrgjxs</t>
+          <t>mjvyxzx</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -3347,7 +3319,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>mnej4gh</t>
+          <t>mn3kzj8</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -3386,7 +3358,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>m2hha3md</t>
+          <t>m2hrfj95</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
@@ -3404,7 +3376,7 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>mkpyjnk</t>
+          <t>mkd0a8o</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -3417,7 +3389,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>mnej4gh</t>
+          <t>mn3kzj8</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -3456,7 +3428,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>m1dytbc5</t>
+          <t>m1dr6xqx</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -3474,7 +3446,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>m1q1h2a</t>
+          <t>m10coly</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -3487,7 +3459,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>molx3s9</t>
+          <t>mokej3l</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -3526,7 +3498,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>m1ezf6tl</t>
+          <t>m1eh07n0</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
@@ -3544,7 +3516,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>m2ymdky</t>
+          <t>m2mu7n0</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -3557,7 +3529,7 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>molx3s9</t>
+          <t>mokej3l</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
@@ -3596,7 +3568,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>m1fuhei2</t>
+          <t>m1fnhmep</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -3614,7 +3586,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>m3ojt68</t>
+          <t>m3vyiil</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -3627,7 +3599,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>molx3s9</t>
+          <t>mokej3l</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -3666,7 +3638,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>m1gbg09v</t>
+          <t>m1gzyern</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
@@ -3684,7 +3656,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>m4bo71q</t>
+          <t>m4lqzwv</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -3697,7 +3669,7 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>molx3s9</t>
+          <t>mokej3l</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
@@ -3736,7 +3708,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>m1hob8o5</t>
+          <t>m1h437ft</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -3754,7 +3726,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>m5o80zg</t>
+          <t>m57wr9j</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -3767,7 +3739,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>molx3s9</t>
+          <t>mokej3l</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -3806,7 +3778,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>m1ic82b2</t>
+          <t>m1ifbovy</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
@@ -3824,7 +3796,7 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>m6bxcak</t>
+          <t>m6tp9v4</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -3837,7 +3809,7 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>molx3s9</t>
+          <t>mokej3l</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -3876,7 +3848,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>m1jnommb</t>
+          <t>m1jz610q</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -3894,7 +3866,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>m7n4lou</t>
+          <t>m7j6k35</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -3907,7 +3879,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>molx3s9</t>
+          <t>mokej3l</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -3946,7 +3918,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>m1kh8znw</t>
+          <t>m1k862ob</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
@@ -3964,7 +3936,7 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>m8bd8ds</t>
+          <t>m8hz0u0</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -3977,7 +3949,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>molx3s9</t>
+          <t>mokej3l</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -4016,7 +3988,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>m1lm1688</t>
+          <t>m1lxyrmf</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -4034,7 +4006,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>m9ka5wa</t>
+          <t>m9obd0s</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -4047,7 +4019,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>molx3s9</t>
+          <t>mokej3l</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -4086,7 +4058,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>m1mki8he</t>
+          <t>m1mhlg5w</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
@@ -4104,7 +4076,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>ma2rn1e</t>
+          <t>mawsv08</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -4117,7 +4089,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>molx3s9</t>
+          <t>mokej3l</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -4156,7 +4128,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>m1ncllv8</t>
+          <t>m1n19two</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -4174,7 +4146,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>mbkzgv3</t>
+          <t>mbpy3qx</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -4187,7 +4159,7 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>molx3s9</t>
+          <t>mokej3l</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -4226,7 +4198,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>m1obid1s</t>
+          <t>m1oveesm</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
@@ -4244,7 +4216,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>mcbd3eq</t>
+          <t>mc7puqh</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -4257,7 +4229,7 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>molx3s9</t>
+          <t>mokej3l</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
@@ -4296,7 +4268,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>m1puwt0d</t>
+          <t>m1p35ggl</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -4314,7 +4286,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>md9qr7l</t>
+          <t>mdu2xvh</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -4327,7 +4299,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>molx3s9</t>
+          <t>mokej3l</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -4366,7 +4338,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>m1qhlqjr</t>
+          <t>m1qep4n6</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
@@ -4384,7 +4356,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>me7wzce</t>
+          <t>me3xemz</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -4397,7 +4369,7 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>molx3s9</t>
+          <t>mokej3l</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
@@ -4436,7 +4408,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>m1rlke9o</t>
+          <t>m1r1i9a1</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -4454,7 +4426,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>mfwnv66</t>
+          <t>mfannts</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -4467,7 +4439,7 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>molx3s9</t>
+          <t>mokej3l</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -4506,7 +4478,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>m1soawcy</t>
+          <t>m1selein</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
@@ -4524,7 +4496,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>mgi1yel</t>
+          <t>mgmpkn5</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -4537,7 +4509,7 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>molx3s9</t>
+          <t>mokej3l</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
@@ -4576,7 +4548,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>m1tthiya</t>
+          <t>m1tk195i</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -4594,7 +4566,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>mhbbnvy</t>
+          <t>mhtq606</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -4607,7 +4579,7 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>molx3s9</t>
+          <t>mokej3l</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
@@ -4646,7 +4618,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>m1uyhtpt</t>
+          <t>m1uahtuw</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
@@ -4664,7 +4636,7 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>miwyf2z</t>
+          <t>miofm01</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -4677,7 +4649,7 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>molx3s9</t>
+          <t>mokej3l</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
@@ -4716,7 +4688,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>m1vn7u79</t>
+          <t>m1v575av</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -4734,7 +4706,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>mjrgjxs</t>
+          <t>mjvyxzx</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -4747,7 +4719,7 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>molx3s9</t>
+          <t>mokej3l</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
@@ -4786,7 +4758,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>m1wn1fdj</t>
+          <t>m1w7utyh</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
@@ -4804,7 +4776,7 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>mkpyjnk</t>
+          <t>mkd0a8o</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -4817,7 +4789,7 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>molx3s9</t>
+          <t>mokej3l</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
@@ -4856,7 +4828,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>msu9wlh</t>
+          <t>msd33sj</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -4874,7 +4846,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>m1q1h2a</t>
+          <t>m10coly</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -4887,7 +4859,7 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>mp30vbe</t>
+          <t>mpe6o5u</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
@@ -4926,7 +4898,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>mtuf1jo</t>
+          <t>mtstkoz</t>
         </is>
       </c>
       <c r="B47" s="2" t="n">
@@ -4944,7 +4916,7 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>m2ymdky</t>
+          <t>m2mu7n0</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -4957,7 +4929,7 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>mp30vbe</t>
+          <t>mpe6o5u</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
@@ -4996,7 +4968,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>mu8ynze</t>
+          <t>muigl61</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -5014,7 +4986,7 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>m3ojt68</t>
+          <t>m3vyiil</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -5027,7 +4999,7 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>mp30vbe</t>
+          <t>mpe6o5u</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
@@ -5066,7 +5038,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>mv5393f</t>
+          <t>mv3ago3</t>
         </is>
       </c>
       <c r="B49" s="2" t="n">
@@ -5084,7 +5056,7 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>m4bo71q</t>
+          <t>m4lqzwv</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -5097,7 +5069,7 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>mp30vbe</t>
+          <t>mpe6o5u</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
@@ -5136,7 +5108,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>mw30w8a</t>
+          <t>mws6w6n</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -5154,7 +5126,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>m5o80zg</t>
+          <t>m57wr9j</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -5167,7 +5139,7 @@
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>mp30vbe</t>
+          <t>mpe6o5u</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
@@ -5206,7 +5178,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>mxccawd</t>
+          <t>mx9ykx1</t>
         </is>
       </c>
       <c r="B51" s="2" t="n">
@@ -5224,7 +5196,7 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>m6bxcak</t>
+          <t>m6tp9v4</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -5237,7 +5209,7 @@
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>mp30vbe</t>
+          <t>mpe6o5u</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
@@ -5276,7 +5248,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>my4osin</t>
+          <t>myvrvhv</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -5294,7 +5266,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>m7n4lou</t>
+          <t>m7j6k35</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -5307,7 +5279,7 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>mp30vbe</t>
+          <t>mpe6o5u</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
@@ -5346,7 +5318,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>mz83oo8</t>
+          <t>mzajdvb</t>
         </is>
       </c>
       <c r="B53" s="2" t="n">
@@ -5364,7 +5336,7 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>m8bd8ds</t>
+          <t>m8hz0u0</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -5377,7 +5349,7 @@
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>mp30vbe</t>
+          <t>mpe6o5u</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
@@ -5416,7 +5388,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>m10qnsh1</t>
+          <t>m10zuxh3</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -5434,7 +5406,7 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>m9ka5wa</t>
+          <t>m9obd0s</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -5447,7 +5419,7 @@
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>mp30vbe</t>
+          <t>mpe6o5u</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
@@ -5486,7 +5458,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>m117uozz</t>
+          <t>m11n7b6t</t>
         </is>
       </c>
       <c r="B55" s="2" t="n">
@@ -5504,7 +5476,7 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>ma2rn1e</t>
+          <t>mawsv08</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
@@ -5517,7 +5489,7 @@
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>mp30vbe</t>
+          <t>mpe6o5u</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
@@ -5556,7 +5528,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>m12r6s7z</t>
+          <t>m12d6b41</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -5574,7 +5546,7 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>mbkzgv3</t>
+          <t>mbpy3qx</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -5587,7 +5559,7 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>mp30vbe</t>
+          <t>mpe6o5u</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
@@ -5626,7 +5598,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>m13tcq83</t>
+          <t>m13l0wyd</t>
         </is>
       </c>
       <c r="B57" s="2" t="n">
@@ -5644,7 +5616,7 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>mcbd3eq</t>
+          <t>mc7puqh</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -5657,7 +5629,7 @@
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>mp30vbe</t>
+          <t>mpe6o5u</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
@@ -5696,7 +5668,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>m14mug0y</t>
+          <t>m14cjeb8</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -5714,7 +5686,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>md9qr7l</t>
+          <t>mdu2xvh</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -5727,7 +5699,7 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>mp30vbe</t>
+          <t>mpe6o5u</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
@@ -5766,7 +5738,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>m15sticr</t>
+          <t>m152hayv</t>
         </is>
       </c>
       <c r="B59" s="2" t="n">
@@ -5784,7 +5756,7 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>me7wzce</t>
+          <t>me3xemz</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
@@ -5797,7 +5769,7 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>mp30vbe</t>
+          <t>mpe6o5u</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
@@ -5836,7 +5808,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>m16stvg3</t>
+          <t>m16lxavj</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -5854,7 +5826,7 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>mfwnv66</t>
+          <t>mfannts</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -5867,7 +5839,7 @@
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>mp30vbe</t>
+          <t>mpe6o5u</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
@@ -5906,7 +5878,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>m17q406v</t>
+          <t>m17g7b8e</t>
         </is>
       </c>
       <c r="B61" s="2" t="n">
@@ -5924,7 +5896,7 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>mgi1yel</t>
+          <t>mgmpkn5</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
@@ -5937,7 +5909,7 @@
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>mp30vbe</t>
+          <t>mpe6o5u</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
@@ -5976,7 +5948,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>m187x4uq</t>
+          <t>m18xzm4s</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -5994,7 +5966,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>mhbbnvy</t>
+          <t>mhtq606</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -6007,7 +5979,7 @@
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>mp30vbe</t>
+          <t>mpe6o5u</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
@@ -6046,7 +6018,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>m19hl4k2</t>
+          <t>m19gf8h8</t>
         </is>
       </c>
       <c r="B63" s="2" t="n">
@@ -6064,7 +6036,7 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>miwyf2z</t>
+          <t>miofm01</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -6077,7 +6049,7 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>mp30vbe</t>
+          <t>mpe6o5u</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
@@ -6116,7 +6088,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>m1arsgmi</t>
+          <t>m1azvubm</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -6134,7 +6106,7 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>mjrgjxs</t>
+          <t>mjvyxzx</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -6147,7 +6119,7 @@
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>mp30vbe</t>
+          <t>mpe6o5u</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
@@ -6186,7 +6158,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>m1bby9ge</t>
+          <t>m1b1k0yz</t>
         </is>
       </c>
       <c r="B65" s="2" t="n">
@@ -6204,7 +6176,7 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>mkpyjnk</t>
+          <t>mkd0a8o</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -6217,7 +6189,7 @@
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>mp30vbe</t>
+          <t>mpe6o5u</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
@@ -6310,7 +6282,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>m1xcpbud</t>
+          <t>m1xv50ed</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -6323,7 +6295,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>mnej4gh</t>
+          <t>mn3kzj8</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -6338,7 +6310,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>m1c0pll0</t>
+          <t>m1cpk8xs</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
@@ -6351,7 +6323,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>molx3s9</t>
+          <t>mokej3l</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -6366,7 +6338,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>mrp14ey</t>
+          <t>mr3vrnc</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -6379,7 +6351,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>mp30vbe</t>
+          <t>mpe6o5u</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -6460,12 +6432,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>m1xcpbud</t>
+          <t>m1xv50ed</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>m1q1h2a</t>
+          <t>m10coly</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -6490,12 +6462,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>m1xcpbud</t>
+          <t>m1xv50ed</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>m2ymdky</t>
+          <t>m2mu7n0</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -6520,12 +6492,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>m1xcpbud</t>
+          <t>m1xv50ed</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>m3ojt68</t>
+          <t>m3vyiil</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -6550,12 +6522,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>m1xcpbud</t>
+          <t>m1xv50ed</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>m4bo71q</t>
+          <t>m4lqzwv</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -6580,12 +6552,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>m1xcpbud</t>
+          <t>m1xv50ed</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>m5o80zg</t>
+          <t>m57wr9j</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -6610,12 +6582,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>m1xcpbud</t>
+          <t>m1xv50ed</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>m6bxcak</t>
+          <t>m6tp9v4</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -6640,12 +6612,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>m1xcpbud</t>
+          <t>m1xv50ed</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>m7n4lou</t>
+          <t>m7j6k35</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -6670,12 +6642,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>m1xcpbud</t>
+          <t>m1xv50ed</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>m8bd8ds</t>
+          <t>m8hz0u0</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -6700,12 +6672,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>m1xcpbud</t>
+          <t>m1xv50ed</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>m9ka5wa</t>
+          <t>m9obd0s</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -6730,12 +6702,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>m1xcpbud</t>
+          <t>m1xv50ed</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>ma2rn1e</t>
+          <t>mawsv08</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -6760,12 +6732,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>m1xcpbud</t>
+          <t>m1xv50ed</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>mbkzgv3</t>
+          <t>mbpy3qx</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -6790,12 +6762,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>m1xcpbud</t>
+          <t>m1xv50ed</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>mcbd3eq</t>
+          <t>mc7puqh</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -6820,12 +6792,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>m1xcpbud</t>
+          <t>m1xv50ed</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>md9qr7l</t>
+          <t>mdu2xvh</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -6850,12 +6822,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>m1xcpbud</t>
+          <t>m1xv50ed</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>me7wzce</t>
+          <t>me3xemz</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -6880,12 +6852,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>m1xcpbud</t>
+          <t>m1xv50ed</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>mfwnv66</t>
+          <t>mfannts</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -6910,12 +6882,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>m1xcpbud</t>
+          <t>m1xv50ed</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>mgi1yel</t>
+          <t>mgmpkn5</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -6940,12 +6912,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>m1xcpbud</t>
+          <t>m1xv50ed</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>mhbbnvy</t>
+          <t>mhtq606</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -6970,12 +6942,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>m1xcpbud</t>
+          <t>m1xv50ed</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>miwyf2z</t>
+          <t>miofm01</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -7000,12 +6972,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>m1xcpbud</t>
+          <t>m1xv50ed</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>mjrgjxs</t>
+          <t>mjvyxzx</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -7030,12 +7002,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>m1xcpbud</t>
+          <t>m1xv50ed</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>mkpyjnk</t>
+          <t>mkd0a8o</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -7060,12 +7032,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>m1c0pll0</t>
+          <t>m1cpk8xs</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>m1q1h2a</t>
+          <t>m10coly</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -7090,12 +7062,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>m1c0pll0</t>
+          <t>m1cpk8xs</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>m2ymdky</t>
+          <t>m2mu7n0</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -7120,12 +7092,12 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>m1c0pll0</t>
+          <t>m1cpk8xs</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>m3ojt68</t>
+          <t>m3vyiil</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -7150,12 +7122,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>m1c0pll0</t>
+          <t>m1cpk8xs</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>m4bo71q</t>
+          <t>m4lqzwv</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -7180,12 +7152,12 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>m1c0pll0</t>
+          <t>m1cpk8xs</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>m5o80zg</t>
+          <t>m57wr9j</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -7210,12 +7182,12 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>m1c0pll0</t>
+          <t>m1cpk8xs</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>m6bxcak</t>
+          <t>m6tp9v4</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -7240,12 +7212,12 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>m1c0pll0</t>
+          <t>m1cpk8xs</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>m7n4lou</t>
+          <t>m7j6k35</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -7270,12 +7242,12 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>m1c0pll0</t>
+          <t>m1cpk8xs</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>m8bd8ds</t>
+          <t>m8hz0u0</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -7300,12 +7272,12 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>m1c0pll0</t>
+          <t>m1cpk8xs</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>m9ka5wa</t>
+          <t>m9obd0s</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -7330,12 +7302,12 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>m1c0pll0</t>
+          <t>m1cpk8xs</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>ma2rn1e</t>
+          <t>mawsv08</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -7360,12 +7332,12 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>m1c0pll0</t>
+          <t>m1cpk8xs</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>mbkzgv3</t>
+          <t>mbpy3qx</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -7390,12 +7362,12 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>m1c0pll0</t>
+          <t>m1cpk8xs</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>mcbd3eq</t>
+          <t>mc7puqh</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -7420,12 +7392,12 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>m1c0pll0</t>
+          <t>m1cpk8xs</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>md9qr7l</t>
+          <t>mdu2xvh</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -7450,12 +7422,12 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>m1c0pll0</t>
+          <t>m1cpk8xs</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>me7wzce</t>
+          <t>me3xemz</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -7480,12 +7452,12 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>m1c0pll0</t>
+          <t>m1cpk8xs</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>mfwnv66</t>
+          <t>mfannts</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -7510,12 +7482,12 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>m1c0pll0</t>
+          <t>m1cpk8xs</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>mgi1yel</t>
+          <t>mgmpkn5</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -7540,12 +7512,12 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>m1c0pll0</t>
+          <t>m1cpk8xs</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>mhbbnvy</t>
+          <t>mhtq606</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -7570,12 +7542,12 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>m1c0pll0</t>
+          <t>m1cpk8xs</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>miwyf2z</t>
+          <t>miofm01</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -7600,12 +7572,12 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>m1c0pll0</t>
+          <t>m1cpk8xs</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>mjrgjxs</t>
+          <t>mjvyxzx</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -7630,12 +7602,12 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>m1c0pll0</t>
+          <t>m1cpk8xs</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>mkpyjnk</t>
+          <t>mkd0a8o</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -7660,12 +7632,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>mrp14ey</t>
+          <t>mr3vrnc</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>m1q1h2a</t>
+          <t>m10coly</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -7690,12 +7662,12 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>mrp14ey</t>
+          <t>mr3vrnc</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>m2ymdky</t>
+          <t>m2mu7n0</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -7720,12 +7692,12 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>mrp14ey</t>
+          <t>mr3vrnc</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>m3ojt68</t>
+          <t>m3vyiil</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -7750,12 +7722,12 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>mrp14ey</t>
+          <t>mr3vrnc</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>m4bo71q</t>
+          <t>m4lqzwv</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -7780,12 +7752,12 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>mrp14ey</t>
+          <t>mr3vrnc</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>m5o80zg</t>
+          <t>m57wr9j</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -7810,12 +7782,12 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>mrp14ey</t>
+          <t>mr3vrnc</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>m6bxcak</t>
+          <t>m6tp9v4</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -7840,12 +7812,12 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>mrp14ey</t>
+          <t>mr3vrnc</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>m7n4lou</t>
+          <t>m7j6k35</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -7870,12 +7842,12 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>mrp14ey</t>
+          <t>mr3vrnc</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>m8bd8ds</t>
+          <t>m8hz0u0</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -7900,12 +7872,12 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>mrp14ey</t>
+          <t>mr3vrnc</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>m9ka5wa</t>
+          <t>m9obd0s</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -7930,12 +7902,12 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>mrp14ey</t>
+          <t>mr3vrnc</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>ma2rn1e</t>
+          <t>mawsv08</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -7960,12 +7932,12 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>mrp14ey</t>
+          <t>mr3vrnc</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>mbkzgv3</t>
+          <t>mbpy3qx</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -7990,12 +7962,12 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>mrp14ey</t>
+          <t>mr3vrnc</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>mcbd3eq</t>
+          <t>mc7puqh</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -8020,12 +7992,12 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>mrp14ey</t>
+          <t>mr3vrnc</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>md9qr7l</t>
+          <t>mdu2xvh</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -8050,12 +8022,12 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>mrp14ey</t>
+          <t>mr3vrnc</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>me7wzce</t>
+          <t>me3xemz</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -8080,12 +8052,12 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>mrp14ey</t>
+          <t>mr3vrnc</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>mfwnv66</t>
+          <t>mfannts</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -8110,12 +8082,12 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>mrp14ey</t>
+          <t>mr3vrnc</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>mgi1yel</t>
+          <t>mgmpkn5</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -8140,12 +8112,12 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>mrp14ey</t>
+          <t>mr3vrnc</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>mhbbnvy</t>
+          <t>mhtq606</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -8170,12 +8142,12 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>mrp14ey</t>
+          <t>mr3vrnc</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>miwyf2z</t>
+          <t>miofm01</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -8200,12 +8172,12 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>mrp14ey</t>
+          <t>mr3vrnc</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>mjrgjxs</t>
+          <t>mjvyxzx</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -8230,12 +8202,12 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>mrp14ey</t>
+          <t>mr3vrnc</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>mkpyjnk</t>
+          <t>mkd0a8o</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">

</xml_diff>